<commit_message>
Finished second level.Almost finished the third one
</commit_message>
<xml_diff>
--- a/KingdomDefenseSpreasheet.xlsx
+++ b/KingdomDefenseSpreasheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\TowerDefensePrototype\TowerDefense-Unity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C00C1FE-1E54-44D4-AFA7-1C8152E4E7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBDE743E-A926-4F98-BFC3-DC322AF09F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D6AA1C1-0FBD-47A9-BC68-9F67466061BB}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="80">
   <si>
     <t>Name</t>
   </si>
@@ -168,9 +168,6 @@
     <t>4 Goblins+4 Bandit Scouts</t>
   </si>
   <si>
-    <t>1 Troll(Boss)</t>
-  </si>
-  <si>
     <t>Level 1 Cost</t>
   </si>
   <si>
@@ -250,6 +247,36 @@
   </si>
   <si>
     <t>1/0(Stun Res)</t>
+  </si>
+  <si>
+    <t>8 Goblins</t>
+  </si>
+  <si>
+    <t>12 Wolves</t>
+  </si>
+  <si>
+    <t>6 Bandit Rangers</t>
+  </si>
+  <si>
+    <t>15 Spiders</t>
+  </si>
+  <si>
+    <t>4 Bandit Scouts+ 2 Bandit Elders</t>
+  </si>
+  <si>
+    <t>Total Gold Generated</t>
+  </si>
+  <si>
+    <t>CyclopsNoRes</t>
+  </si>
+  <si>
+    <t>TrollNoRes</t>
+  </si>
+  <si>
+    <t>1 TrollNoRes(Boss)</t>
+  </si>
+  <si>
+    <t>10 Wolves + 1 CyclopsNoRes(Boss)</t>
   </si>
 </sst>
 </file>
@@ -302,7 +329,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -618,7 +645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B25BA88-B43E-40C4-A113-1639984CB6D3}">
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:M59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.44140625" customWidth="1"/>
@@ -627,7 +654,11 @@
     <col min="4" max="4" width="21.77734375" customWidth="1"/>
     <col min="5" max="5" width="31.109375" customWidth="1"/>
     <col min="6" max="6" width="23.109375" customWidth="1"/>
+    <col min="7" max="7" width="26.88671875" customWidth="1"/>
+    <col min="8" max="8" width="25.77734375" customWidth="1"/>
     <col min="9" max="9" width="11.77734375" customWidth="1"/>
+    <col min="13" max="13" width="21.77734375" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -677,7 +708,7 @@
         <v>150</v>
       </c>
       <c r="E2" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -763,19 +794,19 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="2">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="2">
-        <v>8</v>
-      </c>
       <c r="D6" s="2">
-        <v>350</v>
+        <v>2000</v>
       </c>
       <c r="E6" s="2">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -786,19 +817,19 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" s="2">
-        <v>800</v>
+        <v>350</v>
       </c>
       <c r="E7" s="2">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -809,75 +840,69 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2">
         <v>6</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="2">
-        <v>4</v>
-      </c>
       <c r="D8" s="2">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="E8" s="2">
-        <v>60</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C9" s="2">
         <v>4</v>
       </c>
       <c r="D9" s="2">
-        <v>2750</v>
+        <v>2000</v>
       </c>
       <c r="E9" s="2">
-        <v>120</v>
-      </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="2"/>
       <c r="H9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="I9" s="2"/>
-      <c r="J9" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>19</v>
+        <v>76</v>
       </c>
       <c r="C10" s="2">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D10" s="2">
-        <v>300</v>
+        <v>3000</v>
       </c>
       <c r="E10" s="2">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -888,32 +913,28 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C11" s="2">
         <v>4</v>
       </c>
       <c r="D11" s="2">
-        <v>15000</v>
+        <v>2500</v>
       </c>
       <c r="E11" s="2">
-        <v>1000</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I11" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="I11" s="2"/>
       <c r="J11" s="2" t="s">
         <v>14</v>
       </c>
@@ -921,24 +942,22 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C12" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D12" s="2">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="E12" s="2">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F12" s="2"/>
-      <c r="G12" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -946,98 +965,104 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C13" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D13" s="2">
-        <v>750</v>
+        <v>15000</v>
       </c>
       <c r="E13" s="2">
-        <v>30</v>
-      </c>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
+        <v>1000</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="I13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="2"/>
+      <c r="J13" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C14" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D14" s="2">
-        <v>350</v>
+        <v>600</v>
       </c>
       <c r="E14" s="2">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="G14" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H14" s="2"/>
-      <c r="I14" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C15" s="2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D15" s="2">
-        <v>5000</v>
+        <v>750</v>
       </c>
       <c r="E15" s="2">
-        <v>400</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+      <c r="I15" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C16" s="2">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D16" s="2">
-        <v>120</v>
+        <v>350</v>
       </c>
       <c r="E16" s="2">
-        <v>12</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
@@ -1046,170 +1071,217 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C17" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D17" s="2">
-        <v>750</v>
+        <v>5000</v>
       </c>
       <c r="E17" s="2">
-        <v>60</v>
-      </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>400</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="2"/>
       <c r="H17" s="2"/>
-      <c r="I17" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C18" s="2">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D18" s="2">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="E18" s="2">
-        <v>10</v>
-      </c>
-      <c r="F18" s="2"/>
+        <v>12</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+      <c r="I18" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
+        <v>16</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="2">
+        <v>7</v>
+      </c>
+      <c r="D19" s="2">
+        <v>750</v>
+      </c>
+      <c r="E19" s="2">
+        <v>60</v>
+      </c>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
+        <v>17</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="2">
+        <v>18</v>
+      </c>
+      <c r="D20" s="2">
+        <v>100</v>
+      </c>
+      <c r="E20" s="2">
+        <v>10</v>
+      </c>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="B23" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E23" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="H23" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="I23" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J21" s="1" t="s">
+      <c r="J23" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K21" s="1" t="s">
+      <c r="K23" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="1" t="s">
+      <c r="L23" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A22" s="2">
+      <c r="M23" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
         <v>1</v>
       </c>
-      <c r="B22">
+      <c r="B24" s="2">
         <v>200</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G22" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A23" s="2">
-        <v>2</v>
-      </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A24" s="2">
-        <v>3</v>
-      </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
+      <c r="G24" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L24" s="2"/>
+      <c r="M24">
+        <f>(E2*6 + 10*E3 +4*E4+4*E2+4*E4)+B24</f>
+        <v>560</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
-        <v>4</v>
-      </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="B25" s="2">
+        <v>250</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M25">
+        <f>B25+8*E2+12*E20+6*E7+15*E3+4*E4+2*E8+10*E20</f>
+        <v>970</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1222,9 +1294,9 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1237,9 +1309,9 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1252,9 +1324,9 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1267,9 +1339,9 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1282,9 +1354,9 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1297,340 +1369,370 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A32" s="2">
+        <v>9</v>
+      </c>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="2">
+        <v>10</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D33" s="1" t="s">
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="B36" s="2">
+        <v>100</v>
+      </c>
+      <c r="C36" s="2">
+        <v>200</v>
+      </c>
+      <c r="D36" s="2">
+        <v>350</v>
+      </c>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37" s="2">
+        <v>50</v>
+      </c>
+      <c r="C37" s="2">
+        <v>150</v>
+      </c>
+      <c r="D37" s="2">
+        <v>300</v>
+      </c>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38" s="2">
+        <v>150</v>
+      </c>
+      <c r="C38" s="2">
+        <v>300</v>
+      </c>
+      <c r="D38" s="2">
+        <v>500</v>
+      </c>
+      <c r="E38" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B34" s="2">
+      <c r="B41" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F41" s="2"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B42" s="2">
         <v>100</v>
       </c>
-      <c r="C34" s="2">
-        <v>200</v>
-      </c>
-      <c r="D34" s="2">
-        <v>350</v>
-      </c>
-      <c r="E34" s="2"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B35" s="2">
-        <v>50</v>
-      </c>
-      <c r="C35" s="2">
-        <v>150</v>
-      </c>
-      <c r="D35" s="2">
-        <v>300</v>
-      </c>
-      <c r="E35" s="2"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B36" s="2">
-        <v>150</v>
-      </c>
-      <c r="C36" s="2">
-        <v>300</v>
-      </c>
-      <c r="D36" s="2">
-        <v>500</v>
-      </c>
-      <c r="E36" s="2">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F39" s="2"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B40" s="2">
-        <v>60</v>
-      </c>
-      <c r="C40" s="2">
-        <v>11</v>
-      </c>
-      <c r="D40" s="2">
-        <v>2</v>
-      </c>
-      <c r="E40" s="2">
-        <v>0</v>
-      </c>
-      <c r="F40" s="2"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B41" s="2">
-        <v>15</v>
-      </c>
-      <c r="C41" s="2">
-        <v>15</v>
-      </c>
-      <c r="D41" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="E41" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="F41" s="2"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B42" s="2">
-        <v>60</v>
-      </c>
       <c r="C42" s="2">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D42" s="2">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E42" s="2">
         <v>0</v>
       </c>
       <c r="F42" s="2"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B44" s="1" t="s">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" s="2">
+        <v>20</v>
+      </c>
+      <c r="C43" s="2">
+        <v>15</v>
+      </c>
+      <c r="D43" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="E43" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F43" s="2"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" s="2">
+        <v>60</v>
+      </c>
+      <c r="C44" s="2">
+        <v>16</v>
+      </c>
+      <c r="D44" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="E44" s="2">
+        <v>0</v>
+      </c>
+      <c r="F44" s="2"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C46" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="D46" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="E46" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E44" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B45" s="2">
-        <v>150</v>
-      </c>
-      <c r="C45" s="2">
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2">
+        <v>200</v>
+      </c>
+      <c r="C47" s="2">
         <v>13</v>
       </c>
-      <c r="D45" s="2">
-        <v>1.8</v>
-      </c>
-      <c r="E45" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B46" s="2">
-        <v>30</v>
-      </c>
-      <c r="C46" s="2">
-        <v>17</v>
-      </c>
-      <c r="D46" s="2">
-        <v>0.15</v>
-      </c>
-      <c r="E46" s="2">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B47" s="2">
-        <v>150</v>
-      </c>
-      <c r="C47" s="2">
-        <v>18</v>
-      </c>
       <c r="D47" s="2">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="E47" s="2">
         <v>0</v>
       </c>
     </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2">
+        <v>30</v>
+      </c>
+      <c r="C48" s="2">
+        <v>17</v>
+      </c>
+      <c r="D48" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="E48" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B49" s="1" t="s">
+      <c r="A49" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2">
+        <v>150</v>
+      </c>
+      <c r="C49" s="2">
+        <v>18</v>
+      </c>
+      <c r="D49" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="E49" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C51" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="D51" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="E51" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B50" s="2">
-        <v>300</v>
-      </c>
-      <c r="C50" s="2">
-        <v>15</v>
-      </c>
-      <c r="D50" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="E50" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A51" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B51" s="2">
-        <v>60</v>
-      </c>
-      <c r="C51" s="2">
-        <v>19</v>
-      </c>
-      <c r="D51" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="E51" s="2">
-        <v>0.4</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B52" s="2">
         <v>400</v>
       </c>
       <c r="C52" s="2">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D52" s="2">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E52" s="2">
         <v>0</v>
       </c>
     </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B53" s="2">
+        <v>60</v>
+      </c>
+      <c r="C53" s="2">
+        <v>19</v>
+      </c>
+      <c r="D53" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E53" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D54" s="1" t="s">
+      <c r="A54" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B54" s="2">
+        <v>400</v>
+      </c>
+      <c r="C54" s="2">
+        <v>20</v>
+      </c>
+      <c r="D54" s="2">
+        <v>1</v>
+      </c>
+      <c r="E54" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C56" s="1" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A55" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B55" s="2">
-        <v>4</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A56" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D56" s="2" t="s">
+      <c r="D56" s="1" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="2">
+        <v>4</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B57" s="2">
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="2">
         <v>3</v>
       </c>
-      <c r="C57" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>67</v>
+      <c r="C59" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finished level 3 and 4.Will work on adding desert/snow biome next
</commit_message>
<xml_diff>
--- a/KingdomDefenseSpreasheet.xlsx
+++ b/KingdomDefenseSpreasheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\TowerDefensePrototype\TowerDefense-Unity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBDE743E-A926-4F98-BFC3-DC322AF09F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58DBC796-45CA-471E-A218-AD9F1BE66CF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D6AA1C1-0FBD-47A9-BC68-9F67466061BB}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="85">
   <si>
     <t>Name</t>
   </si>
@@ -277,6 +277,21 @@
   </si>
   <si>
     <t>10 Wolves + 1 CyclopsNoRes(Boss)</t>
+  </si>
+  <si>
+    <t>12 Goblins</t>
+  </si>
+  <si>
+    <t>6 Wargs</t>
+  </si>
+  <si>
+    <t>8 Skeletons + 4 Spiders</t>
+  </si>
+  <si>
+    <t>6 Bandit Ranger</t>
+  </si>
+  <si>
+    <t>3 Wargs + 1 Bandit Leader(Boss)</t>
   </si>
 </sst>
 </file>
@@ -654,7 +669,7 @@
     <col min="4" max="4" width="21.77734375" customWidth="1"/>
     <col min="5" max="5" width="31.109375" customWidth="1"/>
     <col min="6" max="6" width="23.109375" customWidth="1"/>
-    <col min="7" max="7" width="26.88671875" customWidth="1"/>
+    <col min="7" max="7" width="34.109375" customWidth="1"/>
     <col min="8" max="8" width="25.77734375" customWidth="1"/>
     <col min="9" max="9" width="11.77734375" customWidth="1"/>
     <col min="13" max="13" width="21.77734375" customWidth="1"/>
@@ -1283,12 +1298,24 @@
       <c r="A26" s="2">
         <v>3</v>
       </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
+      <c r="B26" s="2">
+        <v>300</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>84</v>
+      </c>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>

</xml_diff>

<commit_message>
Finished Desert Levels.Will continue in the "dark forest/magical" theme.
</commit_message>
<xml_diff>
--- a/KingdomDefenseSpreasheet.xlsx
+++ b/KingdomDefenseSpreasheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\TowerDefensePrototype\TowerDefense-Unity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8966597-6CF7-4AB1-922A-5719410D6B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37ED9EED-E6AA-4518-A512-AF663C6C09AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D6AA1C1-0FBD-47A9-BC68-9F67466061BB}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="108">
   <si>
     <t>Name</t>
   </si>
@@ -307,6 +307,60 @@
   </si>
   <si>
     <t>5 Bandit Elder + 10 Skeletons</t>
+  </si>
+  <si>
+    <t>10 Skeletons</t>
+  </si>
+  <si>
+    <t>12 Wargs</t>
+  </si>
+  <si>
+    <t>5 Mages + 10 Spiders</t>
+  </si>
+  <si>
+    <t>5 Mech Spiders + 3 Bandit Elder</t>
+  </si>
+  <si>
+    <t>8 Wargs  + 5 Enemy Archer</t>
+  </si>
+  <si>
+    <t>Troll +Bandit Leader</t>
+  </si>
+  <si>
+    <t>12 Skeletons</t>
+  </si>
+  <si>
+    <t>10 Wargs</t>
+  </si>
+  <si>
+    <t>6 Mages + 10 Goblins</t>
+  </si>
+  <si>
+    <t>6 Mech Spiders + 4 Witches</t>
+  </si>
+  <si>
+    <t>5 Bandit Elder + 6 Wargs</t>
+  </si>
+  <si>
+    <t>2 Bandit Leader + 5 Mages</t>
+  </si>
+  <si>
+    <t>2 Cyclops + 2 TrollNoRes</t>
+  </si>
+  <si>
+    <t>12 Bandit Rangers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Trolls + 12 Goblins </t>
+  </si>
+  <si>
+    <t>10 Mech Spiders + 15 Wargs</t>
+  </si>
+  <si>
+    <t>5 Bandit leader + 4 Mech Spiders</t>
+  </si>
+  <si>
+    <t>6 Trolls + 4 Bandit Leaders + 10 Mech Spiders</t>
   </si>
 </sst>
 </file>
@@ -683,10 +737,10 @@
     <col min="3" max="3" width="27.5546875" customWidth="1"/>
     <col min="4" max="4" width="21.77734375" customWidth="1"/>
     <col min="5" max="5" width="31.109375" customWidth="1"/>
-    <col min="6" max="6" width="23.109375" customWidth="1"/>
-    <col min="7" max="7" width="34.109375" customWidth="1"/>
+    <col min="6" max="6" width="34.21875" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
     <col min="8" max="8" width="25.77734375" customWidth="1"/>
-    <col min="9" max="9" width="11.77734375" customWidth="1"/>
+    <col min="9" max="9" width="32.6640625" customWidth="1"/>
     <col min="13" max="13" width="21.77734375" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
   </cols>
@@ -1367,14 +1421,30 @@
       <c r="A28" s="2">
         <v>5</v>
       </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
+      <c r="B28" s="2">
+        <v>600</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
@@ -1382,14 +1452,30 @@
       <c r="A29" s="2">
         <v>6</v>
       </c>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
+      <c r="B29" s="2">
+        <v>700</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>102</v>
+      </c>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
     </row>
@@ -1397,12 +1483,24 @@
       <c r="A30" s="2">
         <v>7</v>
       </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
+      <c r="B30" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>107</v>
+      </c>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
@@ -1481,7 +1579,7 @@
         <v>200</v>
       </c>
       <c r="D36" s="2">
-        <v>350</v>
+        <v>400</v>
       </c>
       <c r="E36" s="2"/>
     </row>

</xml_diff>

<commit_message>
Added a unlockable slots and finished level 8
</commit_message>
<xml_diff>
--- a/KingdomDefenseSpreasheet.xlsx
+++ b/KingdomDefenseSpreasheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\TowerDefensePrototype\TowerDefense-Unity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37ED9EED-E6AA-4518-A512-AF663C6C09AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F672217-A08E-4148-A35B-BF3FD763DACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D6AA1C1-0FBD-47A9-BC68-9F67466061BB}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="115">
   <si>
     <t>Name</t>
   </si>
@@ -361,6 +361,27 @@
   </si>
   <si>
     <t>6 Trolls + 4 Bandit Leaders + 10 Mech Spiders</t>
+  </si>
+  <si>
+    <t>15 Skeletons + 10 Mages</t>
+  </si>
+  <si>
+    <t>15 Wargs + 5 Bandit Leaders</t>
+  </si>
+  <si>
+    <t>12 Witches + 15 Mech Spiders</t>
+  </si>
+  <si>
+    <t>2 Warrios + 20 Goblins</t>
+  </si>
+  <si>
+    <t>4 Cyclops + 6 Trolls</t>
+  </si>
+  <si>
+    <t>10 Witches + 10 Mages + 10 Bandit Elders</t>
+  </si>
+  <si>
+    <t>3 Warrios + 8 Bandit Leaders + 5 Cyclops</t>
   </si>
 </sst>
 </file>
@@ -735,12 +756,12 @@
     <col min="1" max="1" width="14.44140625" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
     <col min="3" max="3" width="27.5546875" customWidth="1"/>
-    <col min="4" max="4" width="21.77734375" customWidth="1"/>
+    <col min="4" max="4" width="28.6640625" customWidth="1"/>
     <col min="5" max="5" width="31.109375" customWidth="1"/>
     <col min="6" max="6" width="34.21875" customWidth="1"/>
     <col min="7" max="7" width="43.5546875" customWidth="1"/>
-    <col min="8" max="8" width="25.77734375" customWidth="1"/>
-    <col min="9" max="9" width="32.6640625" customWidth="1"/>
+    <col min="8" max="8" width="42.6640625" customWidth="1"/>
+    <col min="9" max="9" width="38.109375" customWidth="1"/>
     <col min="13" max="13" width="21.77734375" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
   </cols>
@@ -1510,14 +1531,30 @@
       <c r="A31" s="2">
         <v>8</v>
       </c>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
+      <c r="B31" s="2">
+        <v>1200</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
     </row>

</xml_diff>